<commit_message>
Round displayed quantities to one decimal in the planning report
Stored values keep full precision; only the Markdown report changes.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HiyyEV1j3SVjWTXfbBVKNS
</commit_message>
<xml_diff>
--- a/generated_example/logistics_forecast.xlsx
+++ b/generated_example/logistics_forecast.xlsx
@@ -1,26 +1,26 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Dashboard" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="README" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Clean_Data" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Weekly_Analysis" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Monthly_Analysis" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Customer_Category_Analysis" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="Inventory_Demand" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="Forecast" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="Forecast_History" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="Forecast_vs_Actual" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet name="Scenario_Analysis" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet name="Recommendations" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet name="Review_Queue" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet name="Audit" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Clean_Data" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Weekly_Analysis" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Monthly_Analysis" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Customer_Category_Analysis" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Inventory_Demand" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Forecast" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Forecast_History" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Forecast_vs_Actual" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scenario_Analysis" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Recommendations" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Review_Queue" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Audit" sheetId="14" state="visible" r:id="rId14"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Dashboard'!$A$1:$C$18</definedName>

</xml_diff>